<commit_message>
Add IAC solenoid pins (3O/B17, 3M/B7), 3rd wire is power not signal
</commit_message>
<xml_diff>
--- a/wiring/miata-rusefi-wiring-pinout.xlsx
+++ b/wiring/miata-rusefi-wiring-pinout.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="252">
   <si>
     <t xml:space="preserve">rusEFI 99-00 Miata - Wiring Reference</t>
   </si>
@@ -502,6 +502,18 @@
     <t xml:space="preserve">BR/W</t>
   </si>
   <si>
+    <t xml:space="preserve">3M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle Air Control Solenoid Secondary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O</t>
+  </si>
+  <si>
     <t xml:space="preserve">3N</t>
   </si>
   <si>
@@ -514,6 +526,18 @@
     <t xml:space="preserve">LG</t>
   </si>
   <si>
+    <t xml:space="preserve">3O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle Air Control Solenoid Primary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V/R</t>
+  </si>
+  <si>
     <t xml:space="preserve">3S</t>
   </si>
   <si>
@@ -553,6 +577,9 @@
     <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
   </si>
   <si>
+    <t xml:space="preserve">IAC solenoid's 3rd wire is +12V power, not a control signal - ties into switched ignition power (can share 1B/A8), no dedicated rusEFI pin needed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Free / Unused Pins</t>
   </si>
   <si>
@@ -634,21 +661,6 @@
     <t xml:space="preserve">External MAP input, unused since on-board MAP is selected</t>
   </si>
   <si>
-    <t xml:space="preserve">B7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VVT1 / Low Side 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low side output, has flyback diode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low Side 3 / Injector 7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Non-Harness rusEFI Internal Pins</t>
   </si>
   <si>
@@ -718,10 +730,7 @@
     <t xml:space="preserve">  - Narrowband O2 heater output</t>
   </si>
   <si>
-    <t xml:space="preserve">  - Idle Solenoid Primary / Secondary output</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - Idle Stepper Dir / Step / Enable</t>
+    <t xml:space="preserve">  - Idle Stepper Dir / Step / Enable - not used, this IAC is solenoid type, not stepper</t>
   </si>
   <si>
     <t xml:space="preserve">  - ETB#1 and ETB#2 (Dir, Control, Disable) - not used, no electronic throttle</t>
@@ -1824,7 +1833,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -2006,9 +2015,44 @@
       </c>
       <c r="E13" s="6"/>
     </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="E14" s="6"/>
+    </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>174</v>
+      <c r="A15" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="E15" s="6"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -2027,7 +2071,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2037,17 +2081,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>20</v>
@@ -2058,34 +2102,34 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="C7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="C8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>37</v>
@@ -2103,16 +2147,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>45</v>
@@ -2121,81 +2165,81 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>14</v>
@@ -2203,35 +2247,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -2260,12 +2282,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2281,21 +2303,21 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -2315,7 +2337,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -2323,177 +2345,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix IAC: single signal wire (3O/B17), power+ground use existing circuits, B7 free again
</commit_message>
<xml_diff>
--- a/wiring/miata-rusefi-wiring-pinout.xlsx
+++ b/wiring/miata-rusefi-wiring-pinout.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="251">
   <si>
     <t xml:space="preserve">rusEFI 99-00 Miata - Wiring Reference</t>
   </si>
@@ -502,163 +502,160 @@
     <t xml:space="preserve">BR/W</t>
   </si>
   <si>
-    <t xml:space="preserve">3M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idle Air Control Solenoid Secondary</t>
+    <t xml:space="preserve">3N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Pump Relay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle Air Control Solenoid (signal; power+ground not on ECU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V/R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 3 (Cyl 4 Seq)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 4 (Cyl 2 Seq)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3W-3Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Injectors 1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B6, B5, B4, B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y/B, V/G, Y/R, Y/G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAC solenoid is 3-pin: 1 signal wire (3O, to B17), plus power (shares 1B/A8 circuit) and ground (Power Ground, not Sensor Ground). Neither needs a dedicated rusEFI pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free / Unused Pins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harness pins confirmed free (from factory diagram spares or now-deleted emissions equipment):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V/Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marked spare on diagram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">status unclear - user first said taken, then listed as freed. Confirm before using</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">taken, do not reuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed free rusEFI board pins (from connector_B/C/D CSVs):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External MAP input, unused since on-board MAP is selected</t>
   </si>
   <si>
     <t xml:space="preserve">B7</t>
   </si>
   <si>
-    <t xml:space="preserve">O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Pump Relay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idle Air Control Solenoid Primary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 3 (Cyl 4 Seq)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 4 (Cyl 2 Seq)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3W-3Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Injectors 1-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B6, B5, B4, B3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y/B, V/G, Y/R, Y/G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAC solenoid's 3rd wire is +12V power, not a control signal - ties into switched ignition power (can share 1B/A8), no dedicated rusEFI pin needed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free / Unused Pins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harness pins confirmed free (from factory diagram spares or now-deleted emissions equipment):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L/O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marked spare on diagram</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">status unclear - user first said taken, then listed as freed. Confirm before using</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">taken, do not reuse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmed free rusEFI board pins (from connector_B/C/D CSVs):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">External MAP input, unused since on-board MAP is selected</t>
+    <t xml:space="preserve">VVT1 / Low Side 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low side output, has flyback diode</t>
   </si>
   <si>
     <t xml:space="preserve">Non-Harness rusEFI Internal Pins</t>
@@ -1833,11 +1830,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
@@ -2030,29 +2027,14 @@
       </c>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E15" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -2071,7 +2053,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2081,17 +2063,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>20</v>
@@ -2102,34 +2084,34 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>37</v>
@@ -2147,16 +2129,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>45</v>
@@ -2165,81 +2147,81 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>14</v>
@@ -2247,13 +2229,24 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>209</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -2282,12 +2275,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2303,21 +2296,21 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>214</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>216</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>217</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -2345,172 +2338,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix CAN tap placement (3U/3V in Plug 3), add Ambient Temp (3J->D9)
</commit_message>
<xml_diff>
--- a/wiring/miata-rusefi-wiring-pinout.xlsx
+++ b/wiring/miata-rusefi-wiring-pinout.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="254">
   <si>
     <t xml:space="preserve">rusEFI 99-00 Miata - Wiring Reference</t>
   </si>
@@ -502,6 +502,18 @@
     <t xml:space="preserve">BR/W</t>
   </si>
   <si>
+    <t xml:space="preserve">3J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambient Temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D9 (MAP label, repurposed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
     <t xml:space="preserve">3N</t>
   </si>
   <si>
@@ -550,6 +562,30 @@
     <t xml:space="preserve">GY/B</t>
   </si>
   <si>
+    <t xml:space="preserve">3U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus High tap - to ESP32 CAN display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD0 (same bus as 1D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus Low tap - to ESP32 CAN display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD1 (same bus as 1L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/Y</t>
+  </si>
+  <si>
     <t xml:space="preserve">3W-3Z</t>
   </si>
   <si>
@@ -577,18 +613,6 @@
     <t xml:space="preserve">Pin</t>
   </si>
   <si>
-    <t xml:space="preserve">3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
     <t xml:space="preserve">1U</t>
   </si>
   <si>
@@ -598,12 +622,6 @@
     <t xml:space="preserve">3Q</t>
   </si>
   <si>
-    <t xml:space="preserve">3U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L/O</t>
-  </si>
-  <si>
     <t xml:space="preserve">1K</t>
   </si>
   <si>
@@ -638,15 +656,6 @@
   </si>
   <si>
     <t xml:space="preserve">Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">External MAP input, unused since on-board MAP is selected</t>
   </si>
   <si>
     <t xml:space="preserve">B7</t>
@@ -1830,7 +1839,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -2027,14 +2036,59 @@
       </c>
       <c r="E14" s="6"/>
     </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="E15" s="6"/>
+    </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
-        <v>178</v>
-      </c>
+      <c r="A16" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>179</v>
+      <c r="A17" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2053,7 +2107,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2063,17 +2117,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>20</v>
@@ -2084,169 +2138,131 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>186</v>
+        <v>37</v>
       </c>
       <c r="C7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>187</v>
+        <v>76</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>188</v>
+        <v>65</v>
       </c>
       <c r="C8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>76</v>
+        <v>199</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="C11" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="6"/>
+        <v>36</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="B19" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>209</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2275,12 +2291,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2296,21 +2312,21 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -2338,172 +2354,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove Rear Diff Temp to free C14 for ETB TPS2, add DBW ETB conversion section (in progress)
</commit_message>
<xml_diff>
--- a/wiring/miata-rusefi-wiring-pinout.xlsx
+++ b/wiring/miata-rusefi-wiring-pinout.xlsx
@@ -12,9 +12,10 @@
     <sheet name="Plug 1" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Plug 2" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Plug 3" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Free Pins" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Non-Harness" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Notes" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="DBW ETB (in progress)" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Free Pins" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Non-Harness" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Notes" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="289">
   <si>
     <t xml:space="preserve">rusEFI 99-00 Miata - Wiring Reference</t>
   </si>
@@ -58,6 +59,12 @@
     <t xml:space="preserve">Miata factory connector 3 (3A-3Z)</t>
   </si>
   <si>
+    <t xml:space="preserve">DBW ETB (in progress)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive-by-wire throttle body conversion - NOT COMPLETE, has open items</t>
+  </si>
+  <si>
     <t xml:space="preserve">Free Pins</t>
   </si>
   <si>
@@ -169,439 +176,538 @@
     <t xml:space="preserve">1J</t>
   </si>
   <si>
-    <t xml:space="preserve">Rear Differential Temp</t>
+    <t xml:space="preserve">(free - was Rear Differential Temp, removed to free C14 for ETB TPS2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus Low (repurposed Data Link Connector wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR/Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternator Field Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY/R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A/C Request Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D10 (A/C Request / BUTTON2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radiator Cooling Fan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A/C Compressor Clutch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral Switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C6 (HALL2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternator Settings: Enabled, smart PID control, control output B18, target 14.0V, PID defaults.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plug 2 (2A - 2P)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not used for wideband - free, reassign if needed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intake Air Temp (IAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wideband O2 signal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D1 (AUX1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehicle Speed Sensor (VSS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engine Coolant Temp (CLT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Knock Sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brake Pressure Transducer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4 (PPS2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-- (empty cavity in stock harness)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camshaft Position (CMP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY/L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensor +5V Power Supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG/R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crankshaft Position (CKP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tachometer Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B13 (Coil 5 label)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G/O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PA15 (SPI3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flex Fuel Sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D5 (FLEX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Low Pressure Sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C15 (AUX3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W/G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oil Pressure Transducer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3 (AUX2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oil Temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D6 (PPS1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plug 3 (3A - 3Z)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3A / 3B / 3C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECU Power Grounds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3 / A4 / C8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B/Y / B/Y / B/L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Throttle Position - becomes ETB Primary TPS with DBW (in progress)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensor Signal Ground</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B/R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 1 (Cyl 1 &amp; 4 Wasted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 2 (Cyl 2 &amp; 3 Wasted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clutch Pedal Switch / Launch Control Activate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D2 (BUTTON1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BR/W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambient Temperature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D9 (MAP label, repurposed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Pump Relay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle Air Control Solenoid (signal; power+ground not on ECU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V/R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 3 (Cyl 4 Seq)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 4 (Cyl 2 Seq)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus High tap - to ESP32 CAN display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD0 (same bus as 1D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus Low tap - to ESP32 CAN display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD1 (same bus as 1L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3W-3Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Injectors 1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B6, B5, B4, B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y/B, V/G, Y/R, Y/G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAC solenoid is 3-pin: 1 signal wire (3O, to B17), plus power (shares 1B/A8 circuit) and ground (Power Ground, not Sensor Ground). Neither needs a dedicated rusEFI pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive-By-Wire ETB Conversion - IN PROGRESS, NOT COMPLETE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Throttle body: Ford ETC module 12C508, connector C1189 (BK).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Throttle Body Connector (confirmed from TB's own connector diagram)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TB Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Circuit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS1 Negative Slope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU-OG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETC Return (ground)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETC Reference (+5V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GN-VT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS2 Positive Slope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YE-VT (18ga)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor + (TACM+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU-GN (18ga)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor - (TACM-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rusEFI-side assignment (partial - see Status column)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS1 (Primary)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">confirmed, reused from stock cable-throttle TPS pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS2 (Secondary)</t>
   </si>
   <si>
     <t xml:space="preserve">C14 (TPS2)</t>
   </si>
   <si>
-    <t xml:space="preserve">-- (empty cavity in stock harness)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAN Bus Low (repurposed Data Link Connector wire)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BR/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alternator Field Control</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A/C Request Input</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D10 (A/C Request / BUTTON2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Radiator Cooling Fan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A/C Compressor Clutch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neutral Switch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C6 (HALL2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alternator Settings: Enabled, smart PID control, control output B18, target 14.0V, PID defaults.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plug 2 (2A - 2P)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not used for wideband - free, reassign if needed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intake Air Temp (IAT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P/L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wideband O2 signal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D1 (AUX1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vehicle Speed Sensor (VSS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engine Coolant Temp (CLT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Knock Sensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brake Pressure Transducer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C4 (PPS2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Camshaft Position (CMP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY/L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensor +5V Power Supply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crankshaft Position (CKP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tachometer Output</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B13 (Coil 5 label)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G/O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EGT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PA15 (SPI3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flex Fuel Sensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D5 (FLEX)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Low Pressure Sensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C15 (AUX3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W/G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oil Pressure Transducer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C3 (AUX2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oil Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D6 (PPS1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plug 3 (3A - 3Z)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3A / 3B / 3C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECU Power Grounds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A3 / A4 / C8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B/Y / B/Y / B/L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Throttle Position (TPS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensor Signal Ground</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 1 (Cyl 1 &amp; 4 Wasted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 2 (Cyl 2 &amp; 3 Wasted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clutch Pedal Switch / Launch Control Activate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D2 (BUTTON1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BR/W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambient Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D9 (MAP label, repurposed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Pump Relay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idle Air Control Solenoid (signal; power+ground not on ECU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 3 (Cyl 4 Seq)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 4 (Cyl 2 Seq)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAN Bus High tap - to ESP32 CAN display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD0 (same bus as 1D)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L/O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAN Bus Low tap - to ESP32 CAN display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD1 (same bus as 1L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3W-3Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Injectors 1-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B6, B5, B4, B3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y/B, V/G, Y/R, Y/G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAC solenoid is 3-pin: 1 signal wire (3O, to B17), plus power (shares 1B/A8 circuit) and ground (Power Ground, not Sensor Ground). Neither needs a dedicated rusEFI pin.</t>
+    <t xml:space="preserve">reserved - freed by removing Rear Diff Temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor driver (DC1_PWM, DC1_DIR, DC1_DIS, OUT_DC1+/-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNKNOWN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not on connector B/C/D CSVs - likely connector A (no data) or find via TunerStudio ETB#1 dropdowns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">may reuse Sensor +5V (C1) or need dedicated ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">may reuse Sensor Signal Ground (C11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still open:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Motor driver pins unknown - need TunerStudio ETB#1 dropdown screenshots or connector_A.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Accelerator pedal position sensor (dual channel) not yet planned - needs 2 more analog inputs, none currently free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - rusEFI requires both TPS1 and TPS2 wired for safety (confirmed decision: wiring both, not just one)</t>
   </si>
   <si>
     <t xml:space="preserve">Free / Unused Pins</t>
@@ -1212,7 +1318,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -1285,6 +1391,14 @@
       </c>
       <c r="B12" s="2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1315,128 +1429,128 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E9" s="6"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E10" s="6"/>
     </row>
@@ -1568,19 +1682,19 @@
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1591,7 +1705,7 @@
         <v>77</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>65</v>
@@ -1684,49 +1798,49 @@
         <v>100</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>49</v>
+        <v>101</v>
       </c>
       <c r="E10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>57</v>
@@ -1735,28 +1849,28 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>61</v>
@@ -1765,13 +1879,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>73</v>
@@ -1780,46 +1894,46 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E19" s="6"/>
     </row>
@@ -1851,80 +1965,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E4" s="6"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>53</v>
@@ -1933,162 +2047,162 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E17" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2107,162 +2221,195 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>197</v>
+      <c r="A7" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" s="6"/>
+        <v>198</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>76</v>
+      <c r="A8" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="6"/>
+        <v>200</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>198</v>
+      <c r="A9" s="6" t="n">
+        <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="6"/>
+        <v>202</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>199</v>
+      <c r="A10" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>36</v>
+        <v>204</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>201</v>
+      <c r="A11" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>36</v>
+        <v>206</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>202</v>
+      <c r="A12" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>36</v>
+        <v>208</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>207</v>
+      <c r="A15" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>14</v>
+      <c r="A18" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>212</v>
+        <v>221</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -2281,54 +2428,163 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>18</v>
+        <v>229</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>217</v>
-      </c>
+        <v>231</v>
+      </c>
+      <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>219</v>
+        <v>39</v>
       </c>
       <c r="C7" s="6"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>247</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2346,6 +2602,71 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C7" s="6"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:A37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2354,172 +2675,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>222</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>223</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>226</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>230</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>231</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>232</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>233</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>234</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>235</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>236</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>237</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>238</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>239</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>240</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>241</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>242</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>243</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>244</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>245</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>246</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>247</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>248</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>249</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>250</v>
+        <v>285</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>251</v>
+        <v>286</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>252</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>253</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete DBW ETB wiring plan with confirmed motor driver pins (A5/A1)
</commit_message>
<xml_diff>
--- a/wiring/miata-rusefi-wiring-pinout.xlsx
+++ b/wiring/miata-rusefi-wiring-pinout.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Plug 1" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Plug 2" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Plug 3" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="DBW ETB (in progress)" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="DBW ETB" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Free Pins" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Non-Harness" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Notes" sheetId="8" state="visible" r:id="rId10"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="286">
   <si>
     <t xml:space="preserve">rusEFI 99-00 Miata - Wiring Reference</t>
   </si>
@@ -59,10 +59,10 @@
     <t xml:space="preserve">Miata factory connector 3 (3A-3Z)</t>
   </si>
   <si>
-    <t xml:space="preserve">DBW ETB (in progress)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drive-by-wire throttle body conversion - NOT COMPLETE, has open items</t>
+    <t xml:space="preserve">DBW ETB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive-by-wire throttle body conversion wiring plan</t>
   </si>
   <si>
     <t xml:space="preserve">Free Pins</t>
@@ -608,13 +608,13 @@
     <t xml:space="preserve">IAC solenoid is 3-pin: 1 signal wire (3O, to B17), plus power (shares 1B/A8 circuit) and ground (Power Ground, not Sensor Ground). Neither needs a dedicated rusEFI pin.</t>
   </si>
   <si>
-    <t xml:space="preserve">Drive-By-Wire ETB Conversion - IN PROGRESS, NOT COMPLETE</t>
+    <t xml:space="preserve">Drive-By-Wire ETB Conversion</t>
   </si>
   <si>
     <t xml:space="preserve">Throttle body: Ford ETC module 12C508, connector C1189 (BK).</t>
   </si>
   <si>
-    <t xml:space="preserve">Throttle Body Connector (confirmed from TB's own connector diagram)</t>
+    <t xml:space="preserve">Full Wiring Table</t>
   </si>
   <si>
     <t xml:space="preserve">TB Pin</t>
@@ -629,85 +629,76 @@
     <t xml:space="preserve">TPS1 Negative Slope</t>
   </si>
   <si>
+    <t xml:space="preserve">3E (existing wire, reused)</t>
+  </si>
+  <si>
     <t xml:space="preserve">BU-OG</t>
   </si>
   <si>
     <t xml:space="preserve">ETC Return (ground)</t>
   </si>
   <si>
+    <t xml:space="preserve">3F (tap existing)</t>
+  </si>
+  <si>
     <t xml:space="preserve">YE</t>
   </si>
   <si>
     <t xml:space="preserve">ETC Reference (+5V)</t>
   </si>
   <si>
+    <t xml:space="preserve">2I (tap existing)</t>
+  </si>
+  <si>
     <t xml:space="preserve">GN-VT</t>
   </si>
   <si>
     <t xml:space="preserve">TPS2 Positive Slope</t>
   </si>
   <si>
+    <t xml:space="preserve">1J (new wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C14 (TPS2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">YE-VT (18ga)</t>
   </si>
   <si>
     <t xml:space="preserve">Motor + (TACM+)</t>
   </si>
   <si>
+    <t xml:space="preserve">1U (new wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A5 (DC1+ H-Bridge Output)</t>
+  </si>
+  <si>
     <t xml:space="preserve">BU-GN (18ga)</t>
   </si>
   <si>
     <t xml:space="preserve">Motor - (TACM-)</t>
   </si>
   <si>
-    <t xml:space="preserve">rusEFI-side assignment (partial - see Status column)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TPS1 (Primary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">confirmed, reused from stock cable-throttle TPS pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TPS2 (Secondary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C14 (TPS2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reserved - freed by removing Rear Diff Temp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor driver (DC1_PWM, DC1_DIR, DC1_DIS, OUT_DC1+/-)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNKNOWN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not on connector B/C/D CSVs - likely connector A (no data) or find via TunerStudio ETB#1 dropdowns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">may reuse Sensor +5V (C1) or need dedicated ref</t>
-  </si>
-  <si>
-    <t xml:space="preserve">may reuse Sensor Signal Ground (C11)</t>
+    <t xml:space="preserve">3Q (new wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1 (DC1-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed against connector A pinout table (A5=DC1+ H-Bridge Output blue, A1=DC1- white). A3/A4 (grounds) and A7/A8 (vBatt/switched ignition) match what was already in this doc.</t>
   </si>
   <si>
     <t xml:space="preserve">Still open:</t>
   </si>
   <si>
-    <t xml:space="preserve">  - Motor driver pins unknown - need TunerStudio ETB#1 dropdown screenshots or connector_A.csv</t>
-  </si>
-  <si>
     <t xml:space="preserve">  - Accelerator pedal position sensor (dual channel) not yet planned - needs 2 more analog inputs, none currently free</t>
   </si>
   <si>
     <t xml:space="preserve">  - rusEFI requires both TPS1 and TPS2 wired for safety (confirmed decision: wiring both, not just one)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - TunerStudio setup not yet done: set ETB#1 pins, TPS1/TPS2 inputs, run ETB auto-calibrate per rusEFI's Electronic Throttle Body guide</t>
   </si>
   <si>
     <t xml:space="preserve">Free / Unused Pins</t>
@@ -2221,12 +2212,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2254,6 +2247,12 @@
       <c r="C6" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="n">
@@ -2265,16 +2264,28 @@
       <c r="C7" s="6" t="s">
         <v>199</v>
       </c>
+      <c r="D7" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2282,10 +2293,16 @@
         <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>203</v>
+        <v>205</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2293,10 +2310,16 @@
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>205</v>
+        <v>208</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2304,10 +2327,16 @@
         <v>5</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>207</v>
+        <v>212</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2315,101 +2344,41 @@
         <v>6</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>211</v>
+        <v>216</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="B20" s="6" t="s">
+      <c r="A17" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="C20" s="6" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" s="6" t="s">
+    <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>223</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -2438,17 +2407,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>22</v>
@@ -2459,16 +2428,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>39</v>
@@ -2486,7 +2455,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>47</v>
@@ -2495,81 +2464,81 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>16</v>
@@ -2577,13 +2546,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -2612,12 +2581,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2633,21 +2602,21 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -2675,172 +2644,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Discard Ambient Temp (D9/C14 pin conflict + wrong sensor), fix free pins list, warn about CSV reliability
</commit_message>
<xml_diff>
--- a/wiring/miata-rusefi-wiring-pinout.xlsx
+++ b/wiring/miata-rusefi-wiring-pinout.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="282">
   <si>
     <t xml:space="preserve">rusEFI 99-00 Miata - Wiring Reference</t>
   </si>
@@ -506,222 +506,207 @@
     <t xml:space="preserve">BR/W</t>
   </si>
   <si>
+    <t xml:space="preserve">3N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Pump Relay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idle Air Control Solenoid (signal; power+ground not on ECU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V/R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 3 (Cyl 4 Seq)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coil 4 (Cyl 2 Seq)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GY/B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus High tap - to ESP32 CAN display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD0 (same bus as 1D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN Bus Low tap - to ESP32 CAN display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PD1 (same bus as 1L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3W-3Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuel Injectors 1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B6, B5, B4, B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y/B, V/G, Y/R, Y/G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAC solenoid is 3-pin: 1 signal wire (3O, to B17), plus power (shares 1B/A8 circuit) and ground (Power Ground, not Sensor Ground). Neither needs a dedicated rusEFI pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive-By-Wire ETB Conversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Throttle body: Ford ETC module 12C508, connector C1189 (BK).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full Wiring Table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TB Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Circuit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS1 Negative Slope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3E (existing wire, reused)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU-OG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETC Return (ground)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3F (tap existing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETC Reference (+5V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2I (tap existing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GN-VT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPS2 Positive Slope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1J (new wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C14 (TPS2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YE-VT (18ga)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor + (TACM+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1U (new wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A5 (DC1+ H-Bridge Output)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU-GN (18ga)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor - (TACM-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3Q (new wire)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1 (DC1-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed against connector A pinout table (A5=DC1+ H-Bridge Output blue, A1=DC1- white). A3/A4 (grounds) and A7/A8 (vBatt/switched ignition) match what was already in this doc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still open:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Accelerator pedal position sensor (dual channel) not yet planned - needs 2 more analog inputs, none currently free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - rusEFI requires both TPS1 and TPS2 wired for safety (confirmed decision: wiring both, not just one)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - TunerStudio setup not yet done: set ETB#1 pins, TPS1/TPS2 inputs, run ETB auto-calibrate per rusEFI's Electronic Throttle Body guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free / Unused Pins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harness pins confirmed free (from factory diagram spares or now-deleted emissions equipment):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1K</t>
+  </si>
+  <si>
     <t xml:space="preserve">3J</t>
   </si>
   <si>
-    <t xml:space="preserve">Ambient Temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D9 (MAP label, repurposed)</t>
-  </si>
-  <si>
     <t xml:space="preserve">R</t>
   </si>
   <si>
-    <t xml:space="preserve">3N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Pump Relay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idle Air Control Solenoid (signal; power+ground not on ECU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V/R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 3 (Cyl 4 Seq)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coil 4 (Cyl 2 Seq)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GY/B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAN Bus High tap - to ESP32 CAN display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD0 (same bus as 1D)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L/O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAN Bus Low tap - to ESP32 CAN display</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PD1 (same bus as 1L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3W-3Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuel Injectors 1-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B6, B5, B4, B3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y/B, V/G, Y/R, Y/G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grounding rule: keep Power Ground (3A/3B/3C) isolated from Sensor Ground (3F/C11). Do not tie them on the same net.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAC solenoid is 3-pin: 1 signal wire (3O, to B17), plus power (shares 1B/A8 circuit) and ground (Power Ground, not Sensor Ground). Neither needs a dedicated rusEFI pin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drive-By-Wire ETB Conversion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Throttle body: Ford ETC module 12C508, connector C1189 (BK).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full Wiring Table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TB Pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Circuit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TPS1 Negative Slope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3E (existing wire, reused)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BU-OG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ETC Return (ground)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3F (tap existing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ETC Reference (+5V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2I (tap existing)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GN-VT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TPS2 Positive Slope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1J (new wire)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C14 (TPS2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YE-VT (18ga)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor + (TACM+)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1U (new wire)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A5 (DC1+ H-Bridge Output)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BU-GN (18ga)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor - (TACM-)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3Q (new wire)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1 (DC1-)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmed against connector A pinout table (A5=DC1+ H-Bridge Output blue, A1=DC1- white). A3/A4 (grounds) and A7/A8 (vBatt/switched ignition) match what was already in this doc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Still open:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - Accelerator pedal position sensor (dual channel) not yet planned - needs 2 more analog inputs, none currently free</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - rusEFI requires both TPS1 and TPS2 wired for safety (confirmed decision: wiring both, not just one)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - TunerStudio setup not yet done: set ETB#1 pins, TPS1/TPS2 inputs, run ETB auto-calibrate per rusEFI's Electronic Throttle Body guide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free / Unused Pins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harness pins confirmed free (from factory diagram spares or now-deleted emissions equipment):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1U</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V/Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3Q</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1K</t>
-  </si>
-  <si>
     <t xml:space="preserve">3R</t>
   </si>
   <si>
@@ -764,6 +749,9 @@
     <t xml:space="preserve">Low side output, has flyback diode</t>
   </si>
   <si>
+    <t xml:space="preserve">WARNING: TunerStudio caught a real conflict between D9 (labeled MAP) and C14 (labeled TPS2) - both are the same physical MCU pin (PB0), despite being listed as separate connector positions. The connector CSVs and TunerStudio dropdown labels are not fully reliable at the physical-pin level. Treat any pin on this sheet as unconfirmed until it's actually been set and burned without error.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Non-Harness rusEFI Internal Pins</t>
   </si>
   <si>
@@ -791,22 +779,22 @@
     <t xml:space="preserve">Oil Temp Sensor Calibration</t>
   </si>
   <si>
-    <t xml:space="preserve">Sensor: GM / Delphi 25036751 (AC Delco 213-190) thermistor. Input channel D6 (PPS1), harness pin 2P.</t>
+    <t xml:space="preserve">Sensor: ACDelco Gold 213-4514 / 19236568. Input channel D6 (PPS1), harness pin 2P.</t>
   </si>
   <si>
     <t xml:space="preserve">  - Pullup resistor: 2490 ohm</t>
   </si>
   <si>
-    <t xml:space="preserve">  - Lowest temperature: -20 C, Resistance @ LT: 28146 ohm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - Middle temperature: 25 C, Resistance @ MT: 2752 ohm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  - Highest temperature: 100 C, Resistance @ HT: 175.3 ohm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note: values from a third-party source, not independently verified against the GM datasheet. Confirm if oil temp readings look off.</t>
+    <t xml:space="preserve">  - Lowest temperature: -40 C, Resistance @ LT: 100700 ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Middle temperature: 20 C, Resistance @ MT: 2868 ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  - Highest temperature: 100 C, Resistance @ HT: 177 ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: GM 25036751 sensor was originally (incorrectly) used for oil temp - corrected to ACDelco 213-4514. GM part is not currently wired to anything.</t>
   </si>
   <si>
     <t xml:space="preserve">Hardware Notes</t>
@@ -1944,7 +1932,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -2171,29 +2159,14 @@
       </c>
       <c r="E16" s="6"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="E17" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2224,25 +2197,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>20</v>
@@ -2259,13 +2232,13 @@
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>142</v>
@@ -2276,13 +2249,13 @@
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>146</v>
@@ -2293,13 +2266,13 @@
         <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>108</v>
@@ -2310,16 +2283,16 @@
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2327,16 +2300,16 @@
         <v>5</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2344,41 +2317,41 @@
         <v>6</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -2397,7 +2370,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2407,17 +2380,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>22</v>
@@ -2428,76 +2401,78 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>227</v>
+        <v>76</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>228</v>
+        <v>65</v>
       </c>
       <c r="C6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>76</v>
+        <v>224</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>65</v>
+        <v>225</v>
       </c>
       <c r="C8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="6"/>
+        <v>38</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>38</v>
@@ -2506,53 +2481,47 @@
         <v>232</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="B19" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="C19" s="6" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
         <v>240</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -2581,12 +2550,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2602,21 +2571,21 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -2644,172 +2613,172 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>